<commit_message>
Ítem 3b (reunión 2026-09-21): Empresa -> Entidad en toda la app
Renombra User.company a User.entity (migración 0024, también migra field_key de
event_field_configs y las variables de escarapela), acreditación, directorio,
reporte Excel, estadísticas, roster (acepta 'entidad' y 'empresa' legacy) y editor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/templates/plantilla_carga_base_asistentes.xlsx
+++ b/static/templates/plantilla_carga_base_asistentes.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>empresa</t>
+          <t>entidad</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>juan.perez@empresa.com</t>
+          <t>juan.perez@entidad.com</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -723,34 +723,6 @@
           <t>Vegetariano</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -833,12 +805,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>empresa</t>
+          <t>entidad</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Empresa a la que pertenece (opcional).</t>
+          <t>Entidad a la que pertenece (opcional).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ítem 14 (reunión 2026-09-21): Categoría por evento/persona y escarapela distinta por categoría
Categorías definidas por evento en Parámetros (migración 0028); campo Categoría (casillas) en Registrar/Editar
por persona y evento; columna 'categoria' en la carga de base (crea las nuevas) y en el reporte; editor de
escarapelas con 'una para todas' / 'una distinta por categoría'; la impresión usa la plantilla de la categoría.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/templates/plantilla_carga_base_asistentes.xlsx
+++ b/static/templates/plantilla_carga_base_asistentes.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL2"/>
+  <dimension ref="A1:AM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
@@ -523,150 +523,155 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>opcional_1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>opcional_2</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>opcional_3</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>opcional_4</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>opcional_5</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>opcional_6</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>opcional_7</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>opcional_8</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>opcional_9</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>opcional_10</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>opcional_11</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>opcional_12</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>opcional_13</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>opcional_14</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>opcional_15</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>opcional_16</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>opcional_17</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>opcional_18</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>opcional_19</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>opcional_20</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>opcional_21</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>opcional_22</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>opcional_23</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>opcional_24</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>opcional_25</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>opcional_26</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>opcional_27</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>opcional_28</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>opcional_29</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>opcional_30</t>
         </is>
@@ -715,10 +720,15 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>VIP, Prensa</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Talla M</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Vegetariano</t>
         </is>
@@ -735,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -918,6 +928,18 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Categoría(s) del asistente en este evento (opcional). Varias separadas por coma. Las que el evento no tenga se crean solas.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>